<commit_message>
top refac to beh
</commit_message>
<xml_diff>
--- a/instructions.xlsx
+++ b/instructions.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Testes\veriroot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9631D21D-A444-406E-AA15-5A3B9E421AE3}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C9BB93-D3E1-460D-AFBD-8BD668ECB4D7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="1" r:id="rId1"/>
     <sheet name="16-bit instruction word" sheetId="2" r:id="rId2"/>
-    <sheet name="specs" sheetId="4" r:id="rId3"/>
-    <sheet name="regs" sheetId="5" r:id="rId4"/>
-    <sheet name="12-bit instruction word" sheetId="3" r:id="rId5"/>
+    <sheet name="12-bit instruction word" sheetId="3" r:id="rId3"/>
+    <sheet name="specs" sheetId="4" r:id="rId4"/>
+    <sheet name="regs" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -383,7 +383,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -903,13 +903,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -919,10 +916,11 @@
     <xf numFmtId="0" fontId="17" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="17" fillId="33" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -937,12 +935,7 @@
     <xf numFmtId="0" fontId="17" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="17" fillId="33" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1310,7 +1303,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1596,7 +1589,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AC83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1606,52 +1599,52 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
-      <c r="B1" s="4">
+      <c r="B1" s="3">
         <v>15</v>
       </c>
-      <c r="C1" s="4">
+      <c r="C1" s="3">
         <v>14</v>
       </c>
-      <c r="D1" s="4">
+      <c r="D1" s="3">
         <v>13</v>
       </c>
-      <c r="E1" s="4">
+      <c r="E1" s="3">
         <v>12</v>
       </c>
-      <c r="F1" s="4">
+      <c r="F1" s="3">
         <v>11</v>
       </c>
-      <c r="G1" s="4">
+      <c r="G1" s="3">
         <v>10</v>
       </c>
-      <c r="H1" s="4">
+      <c r="H1" s="3">
         <v>9</v>
       </c>
-      <c r="I1" s="4">
+      <c r="I1" s="3">
         <v>8</v>
       </c>
-      <c r="J1" s="4">
+      <c r="J1" s="3">
         <v>7</v>
       </c>
-      <c r="K1" s="4">
+      <c r="K1" s="3">
         <v>6</v>
       </c>
-      <c r="L1" s="4">
+      <c r="L1" s="3">
         <v>5</v>
       </c>
-      <c r="M1" s="4">
+      <c r="M1" s="3">
         <v>4</v>
       </c>
-      <c r="N1" s="4">
+      <c r="N1" s="3">
         <v>3</v>
       </c>
-      <c r="O1" s="4">
+      <c r="O1" s="3">
         <v>2</v>
       </c>
-      <c r="P1" s="4">
+      <c r="P1" s="3">
         <v>1</v>
       </c>
-      <c r="Q1" s="4">
+      <c r="Q1" s="3">
         <v>0</v>
       </c>
       <c r="S1" s="2" t="s">
@@ -1662,12 +1655,12 @@
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -1688,12 +1681,12 @@
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -1714,124 +1707,124 @@
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="3" t="s">
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="5" t="s">
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="3" t="s">
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="5" t="s">
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="3" t="s">
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="11"/>
+      <c r="O6" s="11"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="11"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="5" t="s">
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="6" t="s">
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="5" t="s">
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
       <c r="J8" s="9" t="s">
         <v>54</v>
       </c>
@@ -1847,18 +1840,18 @@
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="5" t="s">
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
       <c r="J9" s="9" t="s">
         <v>54</v>
       </c>
@@ -1874,59 +1867,59 @@
       <c r="A10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="5" t="s">
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5" t="s">
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5" t="s">
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="5" t="s">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5" t="s">
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5" t="s">
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
     </row>
     <row r="12" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2004,12 +1997,16 @@
     <row r="83" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="J8:Q8"/>
-    <mergeCell ref="J9:Q9"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="N10:Q10"/>
-    <mergeCell ref="J11:M11"/>
-    <mergeCell ref="N11:Q11"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="F10:I10"/>
@@ -2021,514 +2018,19 @@
     <mergeCell ref="J6:Q6"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="J7:Q7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="J9:Q9"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="J11:M11"/>
+    <mergeCell ref="N11:Q11"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B1" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="15">
-        <v>1</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" s="16">
-        <v>2</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="16">
-        <v>3</v>
-      </c>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B7" s="16">
-        <v>5</v>
-      </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8" s="16">
-        <v>6</v>
-      </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" s="16">
-        <v>7</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="B10" s="16">
-        <v>8</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="B11" s="16">
-        <v>9</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <ignoredErrors>
-    <ignoredError sqref="B2:B17" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="5" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="15">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="16">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" s="16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" s="16">
-        <v>5</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" s="16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="16">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" s="16">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B11" s="16">
-        <v>9</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AA23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2538,40 +2040,40 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
-      <c r="B1" s="4">
+      <c r="B1" s="3">
         <v>11</v>
       </c>
-      <c r="C1" s="4">
+      <c r="C1" s="3">
         <v>10</v>
       </c>
-      <c r="D1" s="4">
+      <c r="D1" s="3">
         <v>9</v>
       </c>
-      <c r="E1" s="4">
+      <c r="E1" s="3">
         <v>8</v>
       </c>
-      <c r="F1" s="4">
+      <c r="F1" s="3">
         <v>7</v>
       </c>
-      <c r="G1" s="4">
+      <c r="G1" s="3">
         <v>6</v>
       </c>
-      <c r="H1" s="4">
+      <c r="H1" s="3">
         <v>5</v>
       </c>
-      <c r="I1" s="4">
+      <c r="I1" s="3">
         <v>4</v>
       </c>
-      <c r="J1" s="4">
+      <c r="J1" s="3">
         <v>3</v>
       </c>
-      <c r="K1" s="4">
+      <c r="K1" s="3">
         <v>2</v>
       </c>
-      <c r="L1" s="4">
+      <c r="L1" s="3">
         <v>1</v>
       </c>
-      <c r="M1" s="4">
+      <c r="M1" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2579,12 +2081,12 @@
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -2598,12 +2100,12 @@
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -2617,107 +2119,107 @@
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="3" t="s">
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="5" t="s">
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="3" t="s">
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="5" t="s">
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="3" t="s">
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="5" t="s">
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="6" t="s">
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="5" t="s">
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
       <c r="I8" s="9" t="s">
         <v>60</v>
       </c>
@@ -2730,17 +2232,17 @@
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="5" t="s">
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
       <c r="I9" s="9" t="s">
         <v>60</v>
       </c>
@@ -2753,22 +2255,22 @@
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="5" t="s">
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5" t="s">
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
@@ -2776,22 +2278,22 @@
       <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="5" t="s">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5" t="s">
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
     </row>
@@ -2799,22 +2301,22 @@
       <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="5" t="s">
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5" t="s">
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
@@ -2822,22 +2324,22 @@
       <c r="A13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="5" t="s">
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5" t="s">
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
     </row>
@@ -2853,15 +2355,12 @@
     <row r="23" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="I7:M7"/>
-    <mergeCell ref="I8:M8"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="F4:M4"/>
+    <mergeCell ref="B5:E5"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="I5:M5"/>
@@ -2878,13 +2377,485 @@
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="F4:M4"/>
-    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="I7:M7"/>
+    <mergeCell ref="I8:M8"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I13:K13"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="7">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="8">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="8">
+        <v>7</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="8">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="11"/>
+      <c r="F10" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" s="8">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="11"/>
+      <c r="F11" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="12"/>
+      <c r="F12" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="9"/>
+      <c r="F13" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="9"/>
+      <c r="E14" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="C9:E9"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="B2:B17" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="7">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="8">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="8">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="8">
+        <v>9</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>